<commit_message>
Add World Heritage sites
</commit_message>
<xml_diff>
--- a/Table/Place.xlsx
+++ b/Table/Place.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yasuikiyoshi/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yasuikiyoshi/Desktop/My HP/Table/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B573EEB-2F1A-D74B-B708-CAE47D48F989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F924DA-0FB2-0F40-9E87-D1E449F199AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2940" yWindow="2060" windowWidth="28300" windowHeight="17360" xr2:uid="{65BA54D8-9F8C-0F46-8EDF-679078B41DE6}"/>
   </bookViews>
@@ -39,13 +39,31 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t xml:space="preserve">P000001  </t>
-    <phoneticPr fontId="2"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ドリーム合衆国</t>
+  </si>
+  <si>
+    <t>P000002</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>P000003</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>P000001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リアンド</t>
+  </si>
+  <si>
+    <t>道の駅 夕陽が丘そとめ</t>
+  </si>
+  <si>
+    <t>P010001</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -62,15 +80,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="6"/>
       <name val="游ゴシック"/>
       <family val="2"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
@@ -101,7 +121,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -438,19 +458,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79BCB196-AC93-C849-8E7E-C624A14E12D5}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>